<commit_message>
Sprint 1 stand up meeting 1 report added with one day delay
</commit_message>
<xml_diff>
--- a/docs/scrum/Product_Backlog.xlsx
+++ b/docs/scrum/Product_Backlog.xlsx
@@ -86,7 +86,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -112,6 +112,7 @@
     <font>
       <b val="true"/>
       <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Cambria"/>
       <family val="0"/>
       <charset val="1"/>
@@ -122,12 +123,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="11">
@@ -233,7 +228,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -266,15 +261,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -548,7 +539,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16382" style="0" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16382" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -620,7 +611,7 @@
       <c r="A9" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="7" t="s">
         <v>9</v>
       </c>
     </row>
@@ -636,7 +627,7 @@
       <c r="A11" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="8" t="s">
         <v>11</v>
       </c>
     </row>
@@ -644,7 +635,7 @@
       <c r="A12" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="8" t="s">
         <v>12</v>
       </c>
     </row>
@@ -652,7 +643,7 @@
       <c r="A13" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="9" t="s">
         <v>13</v>
       </c>
     </row>
@@ -660,7 +651,7 @@
       <c r="A14" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="11" t="s">
+      <c r="B14" s="10" t="s">
         <v>14</v>
       </c>
     </row>
@@ -668,7 +659,7 @@
       <c r="A15" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="10" t="s">
         <v>15</v>
       </c>
     </row>
@@ -676,7 +667,7 @@
       <c r="A16" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="12" t="s">
+      <c r="B16" s="11" t="s">
         <v>16</v>
       </c>
     </row>
@@ -684,7 +675,7 @@
       <c r="A17" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="12" t="s">
+      <c r="B17" s="11" t="s">
         <v>17</v>
       </c>
     </row>
@@ -692,7 +683,7 @@
       <c r="A18" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="13" t="s">
+      <c r="B18" s="12" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>

<commit_message>
updated for the done items
</commit_message>
<xml_diff>
--- a/docs/scrum/Product_Backlog.xlsx
+++ b/docs/scrum/Product_Backlog.xlsx
@@ -125,7 +125,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -140,20 +140,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF4000"/>
-        <bgColor rgb="FFFF0000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF8000"/>
-        <bgColor rgb="FFFF8080"/>
+        <fgColor rgb="FF81D41A"/>
+        <bgColor rgb="FFACB20C"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFBF00"/>
-        <bgColor rgb="FFACB20C"/>
+        <bgColor rgb="FFFF9900"/>
       </patternFill>
     </fill>
     <fill>
@@ -178,12 +172,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFD4EA6B"/>
         <bgColor rgb="FFBBE33D"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF81D41A"/>
-        <bgColor rgb="FFACB20C"/>
       </patternFill>
     </fill>
   </fills>
@@ -228,7 +216,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -270,14 +258,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -336,8 +316,8 @@
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF81D41A"/>
       <rgbColor rgb="FFFFBF00"/>
-      <rgbColor rgb="FFFF8000"/>
-      <rgbColor rgb="FFFF4000"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
       <rgbColor rgb="FF666699"/>
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF003366"/>
@@ -579,7 +559,7 @@
       <c r="A5" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="5" t="s">
         <v>5</v>
       </c>
     </row>
@@ -587,7 +567,7 @@
       <c r="A6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
     </row>
@@ -595,7 +575,7 @@
       <c r="A7" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="6" t="s">
         <v>7</v>
       </c>
     </row>
@@ -603,7 +583,7 @@
       <c r="A8" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="5" t="s">
         <v>8</v>
       </c>
     </row>
@@ -611,7 +591,7 @@
       <c r="A9" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="5" t="s">
         <v>9</v>
       </c>
     </row>
@@ -619,7 +599,7 @@
       <c r="A10" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -627,7 +607,7 @@
       <c r="A11" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="7" t="s">
         <v>11</v>
       </c>
     </row>
@@ -635,7 +615,7 @@
       <c r="A12" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="7" t="s">
         <v>12</v>
       </c>
     </row>
@@ -643,7 +623,7 @@
       <c r="A13" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -651,7 +631,7 @@
       <c r="A14" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="9" t="s">
         <v>14</v>
       </c>
     </row>
@@ -659,7 +639,7 @@
       <c r="A15" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="9" t="s">
         <v>15</v>
       </c>
     </row>
@@ -667,7 +647,7 @@
       <c r="A16" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="10" t="s">
         <v>16</v>
       </c>
     </row>
@@ -675,7 +655,7 @@
       <c r="A17" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="11" t="s">
+      <c r="B17" s="10" t="s">
         <v>17</v>
       </c>
     </row>
@@ -683,7 +663,7 @@
       <c r="A18" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="12" t="s">
+      <c r="B18" s="5" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>